<commit_message>
Calculated total sales by region and Analyzed total orders by region and Total sales using SUBTOTAL
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AC\Documents\Dmart excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417AAFE4-6E35-424B-9265-D723B7BCD81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84BEDEA-4075-454E-ABE1-EA2B9451A01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,6 +24,7 @@
     <sheet name="Countif_countifs" sheetId="10" r:id="rId9"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet4!$A$18:$A$24</definedName>
     <definedName name="Orders">Dmart_Sales_Data[Order_Id]</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -70,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4198" uniqueCount="665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4224" uniqueCount="679">
   <si>
     <t>Region</t>
   </si>
@@ -2065,6 +2066,48 @@
   </si>
   <si>
     <t>Count Of Sales For Customer Type MEMBER and Payment Mode is UPI and Card</t>
+  </si>
+  <si>
+    <t>Sales_by_North</t>
+  </si>
+  <si>
+    <t>Sales_by_South</t>
+  </si>
+  <si>
+    <t>Sales_by_East</t>
+  </si>
+  <si>
+    <t>Sales_By_West</t>
+  </si>
+  <si>
+    <t>Number of Orders East</t>
+  </si>
+  <si>
+    <t>Number of Order North</t>
+  </si>
+  <si>
+    <t>Number of Order South</t>
+  </si>
+  <si>
+    <t>Number of Order West</t>
+  </si>
+  <si>
+    <t>Total Sales For Year 2023</t>
+  </si>
+  <si>
+    <t>Last 6 Month Sales</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data </t>
+  </si>
+  <si>
+    <t>Total Sales</t>
+  </si>
+  <si>
+    <t>Total Sales Using SUBTOTAL</t>
   </si>
 </sst>
 </file>
@@ -2285,7 +2328,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2349,8 +2392,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -3180,7 +3226,7 @@
     <col min="16" max="16" width="20.08203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="8.6640625" customWidth="1"/>
     <col min="18" max="18" width="68.75" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.75" bestFit="1" customWidth="1"/>
     <col min="20" max="22" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4416,7 +4462,7 @@
         <v>Yes</v>
       </c>
       <c r="Q20" s="1"/>
-      <c r="R20" s="48" t="s">
+      <c r="R20" s="47" t="s">
         <v>659</v>
       </c>
       <c r="S20" s="41">
@@ -4804,7 +4850,7 @@
       <c r="R26" s="47" t="s">
         <v>664</v>
       </c>
-      <c r="S26">
+      <c r="S26" s="29">
         <f>COUNTIFS(Dmart_Sales_Data[customer_type],"Member",Dmart_Sales_Data[payment_mode],"UPI")+COUNTIFS(Dmart_Sales_Data[customer_type],"Member",Dmart_Sales_Data[payment_mode],"Card")</f>
         <v>97</v>
       </c>
@@ -4926,8 +4972,13 @@
         <v>Yes</v>
       </c>
       <c r="Q28" s="1"/>
-      <c r="R28" s="1"/>
-      <c r="S28" s="1"/>
+      <c r="R28" s="47" t="s">
+        <v>665</v>
+      </c>
+      <c r="S28" s="41">
+        <f>SUMIF(Dmart_Sales_Data[Updated_Region],"North",Dmart_Sales_Data[sales])</f>
+        <v>334964.16000000003</v>
+      </c>
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
@@ -4986,8 +5037,13 @@
         <v>No</v>
       </c>
       <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
+      <c r="R29" s="41" t="s">
+        <v>666</v>
+      </c>
+      <c r="S29" s="41">
+        <f>SUMIF(Dmart_Sales_Data[Updated_Region],"South",Dmart_Sales_Data[sales])</f>
+        <v>303623.68999999994</v>
+      </c>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
@@ -5046,8 +5102,13 @@
         <v>Yes</v>
       </c>
       <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
+      <c r="R30" s="41" t="s">
+        <v>667</v>
+      </c>
+      <c r="S30" s="41">
+        <f>SUMIF(Dmart_Sales_Data[Updated_Region],"East",Dmart_Sales_Data[sales])</f>
+        <v>337881.26999999996</v>
+      </c>
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
@@ -5106,8 +5167,13 @@
         <v>No</v>
       </c>
       <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
-      <c r="S31" s="1"/>
+      <c r="R31" s="41" t="s">
+        <v>668</v>
+      </c>
+      <c r="S31" s="41">
+        <f>SUMIF(Dmart_Sales_Data[Updated_Region],"West",Dmart_Sales_Data[sales])</f>
+        <v>346200.06999999983</v>
+      </c>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
@@ -5226,8 +5292,13 @@
         <v>No</v>
       </c>
       <c r="Q33" s="1"/>
-      <c r="R33" s="1"/>
-      <c r="S33" s="1"/>
+      <c r="R33" s="47" t="s">
+        <v>669</v>
+      </c>
+      <c r="S33" s="41">
+        <f>COUNTIF(Dmart_Sales_Data[Updated_Region],"East")</f>
+        <v>125</v>
+      </c>
       <c r="T33" s="1"/>
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
@@ -5286,8 +5357,13 @@
         <v>No</v>
       </c>
       <c r="Q34" s="1"/>
-      <c r="R34" s="1"/>
-      <c r="S34" s="1"/>
+      <c r="R34" s="47" t="s">
+        <v>670</v>
+      </c>
+      <c r="S34" s="41">
+        <f>COUNTIF(Dmart_Sales_Data[Updated_Region],"North")</f>
+        <v>124</v>
+      </c>
       <c r="T34" s="1"/>
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
@@ -5346,8 +5422,13 @@
         <v>No</v>
       </c>
       <c r="Q35" s="1"/>
-      <c r="R35" s="1"/>
-      <c r="S35" s="1"/>
+      <c r="R35" s="47" t="s">
+        <v>671</v>
+      </c>
+      <c r="S35" s="41">
+        <f>COUNTIF(Dmart_Sales_Data[Updated_Region],"South")</f>
+        <v>124</v>
+      </c>
       <c r="T35" s="1"/>
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
@@ -5406,8 +5487,13 @@
         <v>No</v>
       </c>
       <c r="Q36" s="1"/>
-      <c r="R36" s="1"/>
-      <c r="S36" s="1"/>
+      <c r="R36" s="47" t="s">
+        <v>672</v>
+      </c>
+      <c r="S36" s="41">
+        <f>COUNTIF(Dmart_Sales_Data[Updated_Region],"West")</f>
+        <v>125</v>
+      </c>
       <c r="T36" s="1"/>
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
@@ -5526,8 +5612,13 @@
         <v>No</v>
       </c>
       <c r="Q38" s="1"/>
-      <c r="R38" s="1"/>
-      <c r="S38" s="1"/>
+      <c r="R38" s="47" t="s">
+        <v>673</v>
+      </c>
+      <c r="S38" s="41">
+        <f>SUMIF(Dmart_Sales_Data[order_date],"&lt;2024-01-01",Dmart_Sales_Data[sales])</f>
+        <v>654586.69000000018</v>
+      </c>
       <c r="T38" s="1"/>
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
@@ -5586,8 +5677,13 @@
         <v>No</v>
       </c>
       <c r="Q39" s="1"/>
-      <c r="R39" s="1"/>
-      <c r="S39" s="1"/>
+      <c r="R39" s="47" t="s">
+        <v>674</v>
+      </c>
+      <c r="S39" s="41">
+        <f>SUMIF(Dmart_Sales_Data[order_date],"&gt;=2024-07-01",Dmart_Sales_Data[sales])</f>
+        <v>368049.34999999992</v>
+      </c>
       <c r="T39" s="1"/>
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
@@ -5706,8 +5802,13 @@
         <v>Yes</v>
       </c>
       <c r="Q41" s="1"/>
-      <c r="R41" s="1"/>
-      <c r="S41" s="1"/>
+      <c r="R41" s="47" t="s">
+        <v>677</v>
+      </c>
+      <c r="S41" s="41">
+        <f>SUM(Dmart_Sales_Data[sales])</f>
+        <v>1322669.1900000023</v>
+      </c>
       <c r="T41" s="1"/>
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
@@ -5766,8 +5867,13 @@
         <v>No</v>
       </c>
       <c r="Q42" s="1"/>
-      <c r="R42" s="1"/>
-      <c r="S42" s="1"/>
+      <c r="R42" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="S42" s="41">
+        <f>SUBTOTAL(9,Dmart_Sales_Data[sales])</f>
+        <v>1322669.1900000023</v>
+      </c>
       <c r="T42" s="1"/>
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
@@ -5826,8 +5932,6 @@
         <v>Yes</v>
       </c>
       <c r="Q43" s="1"/>
-      <c r="R43" s="1"/>
-      <c r="S43" s="1"/>
       <c r="T43" s="1"/>
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
@@ -33267,8 +33371,13 @@
       <c r="V502" s="1"/>
     </row>
     <row r="503" spans="1:24" ht="14.25" customHeight="1">
-      <c r="A503" s="1"/>
-      <c r="B503" s="2"/>
+      <c r="A503" s="49" t="s">
+        <v>677</v>
+      </c>
+      <c r="B503" s="1">
+        <f>SUM(Dmart_Sales_Data[sales])</f>
+        <v>1322669.1900000023</v>
+      </c>
       <c r="C503" s="2"/>
       <c r="D503" s="1"/>
       <c r="E503" s="1"/>
@@ -33290,9 +33399,14 @@
       <c r="U503" s="1"/>
       <c r="V503" s="1"/>
     </row>
-    <row r="504" spans="1:24" ht="14.25" customHeight="1">
-      <c r="A504" s="1"/>
-      <c r="B504" s="2"/>
+    <row r="504" spans="1:24" ht="12.5" customHeight="1">
+      <c r="A504" s="49" t="s">
+        <v>678</v>
+      </c>
+      <c r="B504" s="1">
+        <f>SUBTOTAL(9,Dmart_Sales_Data[sales])</f>
+        <v>1322669.1900000023</v>
+      </c>
       <c r="C504" s="2"/>
       <c r="D504" s="1"/>
       <c r="E504" s="1"/>
@@ -46267,11 +46381,11 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D841484-71F5-47BE-A450-CBFC991A1C36}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
-    <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.25" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -46364,7 +46478,116 @@
         <v>1200</v>
       </c>
     </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="29" t="s">
+        <v>574</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>579</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="29" t="s">
+        <v>576</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>580</v>
+      </c>
+      <c r="C11" s="29">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="29" t="s">
+        <v>575</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>581</v>
+      </c>
+      <c r="C12" s="29">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="29" t="s">
+        <v>577</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>582</v>
+      </c>
+      <c r="C13" s="29">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="29" t="s">
+        <v>575</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>583</v>
+      </c>
+      <c r="C14" s="29">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="29"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="48" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19">
+        <v>120</v>
+      </c>
+      <c r="C19">
+        <f>SUBTOTAL(9,A19:A24)</f>
+        <v>578</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="C20">
+        <f>SUBTOTAL(1,A19:A24)</f>
+        <v>96.333333333333329</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24">
+        <v>230</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A18:A24" xr:uid="{4D841484-71F5-47BE-A450-CBFC991A1C36}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Used Vlookup and Index-Match functions
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AC\Documents\Dmart excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84BEDEA-4075-454E-ABE1-EA2B9451A01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F93455-6A99-42EA-A4BA-A01DB271CF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DMart_Dataset" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Sheet2" sheetId="7" r:id="rId6"/>
     <sheet name="Sheet4" sheetId="9" r:id="rId7"/>
     <sheet name="Sheet3" sheetId="8" r:id="rId8"/>
-    <sheet name="Countif_countifs" sheetId="10" r:id="rId9"/>
+    <sheet name="LOOKUP_FUNCTION" sheetId="10" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet4!$A$18:$A$24</definedName>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4224" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4242" uniqueCount="683">
   <si>
     <t>Region</t>
   </si>
@@ -2108,6 +2108,18 @@
   </si>
   <si>
     <t>Total Sales Using SUBTOTAL</t>
+  </si>
+  <si>
+    <t>EmpID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EmployeeID </t>
+  </si>
+  <si>
+    <t>UsingVlookup</t>
+  </si>
+  <si>
+    <t>UsingIndex</t>
   </si>
 </sst>
 </file>
@@ -2173,7 +2185,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2213,6 +2225,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2323,12 +2341,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2397,11 +2416,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="27">
     <dxf>
@@ -2461,26 +2483,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2965,6 +2967,26 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2979,27 +3001,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E9EA62CC-89F7-4F3B-BD9F-F8C05C3E138F}" name="Dmart_Sales_Data" displayName="Dmart_Sales_Data" ref="A1:P499" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E9EA62CC-89F7-4F3B-BD9F-F8C05C3E138F}" name="Dmart_Sales_Data" displayName="Dmart_Sales_Data" ref="A1:P499" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" tableBorderDxfId="22">
   <autoFilter ref="A1:P499" xr:uid="{E9EA62CC-89F7-4F3B-BD9F-F8C05C3E138F}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{B7F21A3A-E9F0-468E-97F8-7B3FAC2DBDFE}" name="Order_Id" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{05F6E9FA-25A7-4B6B-A848-54A6D80DECAC}" name="Region" dataDxfId="22"/>
-    <tableColumn id="17" xr3:uid="{C83619D3-C35D-4142-8385-D268D1C83988}" name="Updated_Region" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{5FCC796F-4F4F-493A-B022-58C82C79A93A}" name="Category" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{3FCE68DB-4CEC-40AE-B661-EA53366A51E8}" name="sales" dataDxfId="19"/>
-    <tableColumn id="15" xr3:uid="{6B2115CE-A9BC-4D55-898F-D45A1E013F08}" name="Sales_Range" dataDxfId="18">
+    <tableColumn id="1" xr3:uid="{B7F21A3A-E9F0-468E-97F8-7B3FAC2DBDFE}" name="Order_Id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{05F6E9FA-25A7-4B6B-A848-54A6D80DECAC}" name="Region" dataDxfId="20"/>
+    <tableColumn id="17" xr3:uid="{C83619D3-C35D-4142-8385-D268D1C83988}" name="Updated_Region" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{5FCC796F-4F4F-493A-B022-58C82C79A93A}" name="Category" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{3FCE68DB-4CEC-40AE-B661-EA53366A51E8}" name="sales" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{6B2115CE-A9BC-4D55-898F-D45A1E013F08}" name="Sales_Range" dataDxfId="16">
       <calculatedColumnFormula>IF(Dmart_Sales_Data[[#This Row],[sales]]&lt;1000,"Low_Sales",IF(Dmart_Sales_Data[[#This Row],[sales]]&lt;3000,"mediam_Sales","High_Sales"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{2FAB2D00-DB8F-414F-9E4B-C312F1DABCA6}" name="discount" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{2A898607-8934-4774-A603-6022A491EEB6}" name="quantity" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{B389254D-5FC3-4CBC-AC59-9299E28BC597}" name="order_date" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{8B502A45-B41C-4FC8-9D80-834A966FB61B}" name="delivery_date" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{B8C2A60B-B1ED-4620-85AC-ABEB1CF14605}" name="customer_type" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{0EC10F89-695A-4256-8BA6-B87E50EF1DA5}" name="payment_mode" dataDxfId="12"/>
-    <tableColumn id="12" xr3:uid="{12061CEA-BF50-4634-8511-FAC42B11C1A9}" name="profit" dataDxfId="11"/>
-    <tableColumn id="16" xr3:uid="{33BB5293-65CC-4A1F-8DC0-7511030FFE84}" name="Updated_City" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{F70F69E9-EB53-4CF5-AD04-B968AD862ED3}" name="city" dataDxfId="9"/>
-    <tableColumn id="19" xr3:uid="{5F1422B9-56D4-4E12-9A8B-A83D504A1CD5}" name="Discount_Category" dataDxfId="8">
+    <tableColumn id="10" xr3:uid="{2FAB2D00-DB8F-414F-9E4B-C312F1DABCA6}" name="discount" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{2A898607-8934-4774-A603-6022A491EEB6}" name="quantity" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{B389254D-5FC3-4CBC-AC59-9299E28BC597}" name="order_date" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{8B502A45-B41C-4FC8-9D80-834A966FB61B}" name="delivery_date" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{B8C2A60B-B1ED-4620-85AC-ABEB1CF14605}" name="customer_type" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{0EC10F89-695A-4256-8BA6-B87E50EF1DA5}" name="payment_mode" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{12061CEA-BF50-4634-8511-FAC42B11C1A9}" name="profit" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{33BB5293-65CC-4A1F-8DC0-7511030FFE84}" name="Updated_City" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{F70F69E9-EB53-4CF5-AD04-B968AD862ED3}" name="city" dataDxfId="7"/>
+    <tableColumn id="19" xr3:uid="{5F1422B9-56D4-4E12-9A8B-A83D504A1CD5}" name="Discount_Category" dataDxfId="6">
       <calculatedColumnFormula>IF(AND(Dmart_Sales_Data[[#This Row],[customer_type]]="Member",OR(Dmart_Sales_Data[[#This Row],[payment_mode]]="UPI",Dmart_Sales_Data[[#This Row],[payment_mode]]="Card")),"Yes","No")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -45335,8 +45357,8 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="E1:G1048576">
-    <cfRule type="top10" dxfId="7" priority="2" bottom="1" rank="10"/>
-    <cfRule type="top10" dxfId="6" priority="3" rank="10"/>
+    <cfRule type="top10" dxfId="26" priority="2" bottom="1" rank="10"/>
+    <cfRule type="top10" dxfId="25" priority="3" rank="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="colorScale" priority="1">
@@ -46667,9 +46689,205 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99BD4BA0-200E-4CD2-A5C3-8AB709EAE206}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11.9140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.08203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="34" t="s">
+        <v>679</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>602</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>576</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>627</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="29">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>607</v>
+      </c>
+      <c r="C2" s="29">
+        <v>70000</v>
+      </c>
+      <c r="D2" s="50">
+        <f>IF(C2&gt;=75000,15%,IF(C2&gt;=70000,10%,IF(C2&gt;=50000,5%,IF(C2&lt;=50000,0))))</f>
+        <v>0.1</v>
+      </c>
+      <c r="E2" s="29">
+        <f>C2*D2</f>
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="29">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>608</v>
+      </c>
+      <c r="C3" s="29">
+        <v>50000</v>
+      </c>
+      <c r="D3" s="50">
+        <f t="shared" ref="D3:D6" si="0">IF(C3&gt;=75000,15%,IF(C3&gt;=70000,10%,IF(C3&gt;=50000,5%,IF(C3&lt;=50000,0))))</f>
+        <v>0.05</v>
+      </c>
+      <c r="E3" s="29">
+        <f t="shared" ref="E3:E6" si="1">C3*D3</f>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="29">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>609</v>
+      </c>
+      <c r="C4" s="29">
+        <v>45000</v>
+      </c>
+      <c r="D4" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E4" s="29">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="29">
+        <v>1004</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>610</v>
+      </c>
+      <c r="C5" s="29">
+        <v>75000</v>
+      </c>
+      <c r="D5" s="50">
+        <f t="shared" si="0"/>
+        <v>0.15</v>
+      </c>
+      <c r="E5" s="29">
+        <f t="shared" si="1"/>
+        <v>11250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="29">
+        <v>1005</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>626</v>
+      </c>
+      <c r="C6" s="36">
+        <v>55000</v>
+      </c>
+      <c r="D6" s="50">
+        <f t="shared" si="0"/>
+        <v>0.05</v>
+      </c>
+      <c r="E6" s="29">
+        <f t="shared" si="1"/>
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="51" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="B9" s="38" t="s">
+        <v>680</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>576</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>628</v>
+      </c>
+      <c r="F9">
+        <f>MATCH(B5,B1:B6,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="B10" s="29">
+        <v>1001</v>
+      </c>
+      <c r="C10" s="29">
+        <f>VLOOKUP(B10,A1:E6,MATCH("Sales",A1:E1,0),FALSE)</f>
+        <v>70000</v>
+      </c>
+      <c r="D10" s="29">
+        <f>VLOOKUP(B10,A1:E6,5,FALSE)</f>
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="F11">
+        <f>MATCH("Sales",A1:E1,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="51" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="B13" s="38" t="s">
+        <v>680</v>
+      </c>
+      <c r="C13" s="38" t="s">
+        <v>576</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>628</v>
+      </c>
+      <c r="F13">
+        <f>MATCH(B14,A2:A6,0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="B14">
+        <v>1002</v>
+      </c>
+      <c r="C14">
+        <f>INDEX(A2:E6,MATCH(B14,A2:A6,0),3)</f>
+        <v>50000</v>
+      </c>
+      <c r="D14">
+        <f>INDEX(A2:E6,MATCH(B14,A2:A6,0),5)</f>
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{088DACFA-72EC-47C8-A11D-167B072525C0}">
+      <formula1>$A$2:$A$6</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Learnt Pivot Tables and charts
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AC\Documents\Dmart excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A62201-7043-44DF-9511-0082E7E13B4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283B3B23-46CA-4E60-9BFF-70F68EA8E59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DMart_Dataset" sheetId="1" r:id="rId1"/>
@@ -2170,10 +2170,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -2427,7 +2428,7 @@
     <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2506,13 +2507,18 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -45696,7 +45702,7 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="65" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -45706,7 +45712,7 @@
       <c r="B1" s="38" t="s">
         <v>693</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="63" t="s">
         <v>694</v>
       </c>
       <c r="D1" s="57" t="s">
@@ -45738,7 +45744,7 @@
       <c r="B3" s="29">
         <v>4</v>
       </c>
-      <c r="C3" s="58"/>
+      <c r="C3" s="64"/>
       <c r="D3" s="29">
         <v>49</v>
       </c>
@@ -45750,15 +45756,16 @@
       <c r="B4" s="29">
         <v>3</v>
       </c>
-      <c r="C4" s="58"/>
+      <c r="C4" s="64"/>
       <c r="D4" s="29">
         <v>47</v>
       </c>
+      <c r="F4" s="59"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="29"/>
       <c r="B5" s="29"/>
-      <c r="C5" s="58"/>
+      <c r="C5" s="64"/>
       <c r="D5" s="29">
         <v>75</v>
       </c>

</xml_diff>